<commit_message>
fix: read correctly the inversion
</commit_message>
<xml_diff>
--- a/Input_0.1.xlsx
+++ b/Input_0.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\herna\Desktop\Repos\TecBooks_V2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0152A241-7C3C-44A8-8110-8E3116A546DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{746121D2-7451-44DF-B741-4BD34FCB1C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28800" yWindow="0" windowWidth="14400" windowHeight="15600" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Premisas" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="264">
   <si>
     <t>Producto:</t>
   </si>
@@ -980,7 +980,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -1105,12 +1105,55 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1201,6 +1244,10 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="40" fontId="10" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4617,7 +4664,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:S1000"/>
+  <dimension ref="A1:P1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.109375" customWidth="1"/>
@@ -4628,200 +4675,126 @@
     <col min="7" max="7" width="13.33203125" customWidth="1"/>
     <col min="8" max="8" width="10.6640625" customWidth="1"/>
     <col min="9" max="9" width="22.44140625" customWidth="1"/>
-    <col min="10" max="26" width="10.6640625" customWidth="1"/>
+    <col min="10" max="19" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="26" width="10.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="6" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="6">
         <v>2025</v>
       </c>
-      <c r="D1" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F1" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="G1" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="H1" s="11" t="s">
-        <v>24</v>
+      <c r="C1" s="6">
+        <v>2026</v>
+      </c>
+      <c r="D1" s="6">
+        <v>2027</v>
+      </c>
+      <c r="E1" s="6">
+        <v>2028</v>
+      </c>
+      <c r="F1" s="6">
+        <v>2029</v>
+      </c>
+      <c r="G1" s="6">
+        <v>2030</v>
+      </c>
+      <c r="H1" s="6">
+        <v>2031</v>
       </c>
       <c r="I1" s="6">
-        <v>2025</v>
+        <v>2032</v>
       </c>
       <c r="J1" s="6">
-        <f t="shared" ref="J1:S1" si="0">I1+1</f>
-        <v>2026</v>
+        <v>2033</v>
       </c>
       <c r="K1" s="6">
-        <f t="shared" si="0"/>
-        <v>2027</v>
+        <v>2034</v>
       </c>
       <c r="L1" s="6">
-        <f t="shared" si="0"/>
-        <v>2028</v>
-      </c>
-      <c r="M1" s="6">
-        <f t="shared" si="0"/>
-        <v>2029</v>
-      </c>
-      <c r="N1" s="6">
-        <f t="shared" si="0"/>
-        <v>2030</v>
-      </c>
-      <c r="O1" s="6">
-        <f t="shared" si="0"/>
-        <v>2031</v>
-      </c>
-      <c r="P1" s="6">
-        <f t="shared" si="0"/>
-        <v>2032</v>
-      </c>
-      <c r="Q1" s="6">
-        <f t="shared" si="0"/>
-        <v>2033</v>
-      </c>
-      <c r="R1" s="6">
-        <f t="shared" si="0"/>
-        <v>2034</v>
-      </c>
-      <c r="S1" s="6">
-        <f t="shared" si="0"/>
         <v>2035</v>
       </c>
     </row>
-    <row r="2" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="19" t="s">
         <v>35</v>
       </c>
       <c r="B2" s="20">
         <v>0.8</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" s="21">
-        <v>60</v>
-      </c>
-      <c r="G2" s="21">
-        <v>6</v>
-      </c>
-      <c r="H2" s="21">
-        <f t="shared" ref="H2:H17" si="1">F2/G2</f>
-        <v>10</v>
-      </c>
-      <c r="I2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="J2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="K2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="L2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="M2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="N2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="O2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="P2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="Q2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="R2" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="S2" s="21">
-        <v>2800000</v>
-      </c>
-    </row>
-    <row r="3" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="68">
+        <v>0.85</v>
+      </c>
+      <c r="D2" s="68">
+        <v>0.9</v>
+      </c>
+      <c r="E2" s="68">
+        <v>0.9</v>
+      </c>
+      <c r="F2" s="68">
+        <v>0.9</v>
+      </c>
+      <c r="G2" s="68">
+        <v>0.9</v>
+      </c>
+      <c r="H2" s="68">
+        <v>0.9</v>
+      </c>
+      <c r="I2" s="68">
+        <v>0.9</v>
+      </c>
+      <c r="J2" s="68">
+        <v>0.9</v>
+      </c>
+      <c r="K2" s="68">
+        <v>0.9</v>
+      </c>
+      <c r="L2" s="68">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="23" t="s">
         <v>43</v>
       </c>
       <c r="B3" s="24">
         <v>420</v>
       </c>
-      <c r="D3" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="F3" s="21">
-        <v>12</v>
-      </c>
-      <c r="G3" s="21">
-        <v>1</v>
-      </c>
-      <c r="H3" s="21">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="I3" s="21">
-        <v>2400000</v>
-      </c>
-      <c r="J3" s="21">
-        <f t="shared" ref="J3:S3" si="2">I3</f>
-        <v>2400000</v>
-      </c>
-      <c r="K3" s="21">
-        <f t="shared" si="2"/>
-        <v>2400000</v>
-      </c>
-      <c r="L3" s="21">
-        <f t="shared" si="2"/>
-        <v>2400000</v>
-      </c>
-      <c r="M3" s="21">
-        <f t="shared" si="2"/>
-        <v>2400000</v>
-      </c>
-      <c r="N3" s="21">
-        <f t="shared" si="2"/>
-        <v>2400000</v>
-      </c>
-      <c r="O3" s="21">
-        <f t="shared" si="2"/>
-        <v>2400000</v>
-      </c>
-      <c r="P3" s="21">
-        <f t="shared" si="2"/>
-        <v>2400000</v>
-      </c>
-      <c r="Q3" s="21">
-        <f t="shared" si="2"/>
-        <v>2400000</v>
-      </c>
-      <c r="R3" s="21">
-        <f t="shared" si="2"/>
-        <v>2400000</v>
-      </c>
-      <c r="S3" s="21">
-        <f t="shared" si="2"/>
-        <v>2400000</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C3" s="70">
+        <f>E33</f>
+        <v>40</v>
+      </c>
+      <c r="D3" s="70">
+        <v>40</v>
+      </c>
+      <c r="E3" s="70">
+        <v>40</v>
+      </c>
+      <c r="F3" s="70">
+        <v>40</v>
+      </c>
+      <c r="G3" s="70">
+        <v>40</v>
+      </c>
+      <c r="H3" s="70">
+        <v>40</v>
+      </c>
+      <c r="I3" s="70">
+        <v>40</v>
+      </c>
+      <c r="J3" s="70">
+        <v>40</v>
+      </c>
+      <c r="K3" s="70">
+        <v>40</v>
+      </c>
+      <c r="L3" s="70">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="23" t="s">
         <v>65</v>
       </c>
@@ -4829,469 +4802,267 @@
         <f>3600/B3</f>
         <v>8.5714285714285712</v>
       </c>
-      <c r="D4" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="E4" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="F4" s="21">
-        <v>12</v>
-      </c>
-      <c r="G4" s="21">
-        <v>1</v>
-      </c>
-      <c r="H4" s="21">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="I4" s="21">
-        <v>2000000</v>
-      </c>
-      <c r="J4" s="21">
-        <f t="shared" ref="J4:S4" si="3">I4</f>
-        <v>2000000</v>
-      </c>
-      <c r="K4" s="21">
-        <f t="shared" si="3"/>
-        <v>2000000</v>
-      </c>
-      <c r="L4" s="21">
-        <f t="shared" si="3"/>
-        <v>2000000</v>
-      </c>
-      <c r="M4" s="21">
-        <f t="shared" si="3"/>
-        <v>2000000</v>
-      </c>
-      <c r="N4" s="21">
-        <f t="shared" si="3"/>
-        <v>2000000</v>
-      </c>
-      <c r="O4" s="21">
-        <f t="shared" si="3"/>
-        <v>2000000</v>
-      </c>
-      <c r="P4" s="21">
-        <f t="shared" si="3"/>
-        <v>2000000</v>
-      </c>
-      <c r="Q4" s="21">
-        <f t="shared" si="3"/>
-        <v>2000000</v>
-      </c>
-      <c r="R4" s="21">
-        <f t="shared" si="3"/>
-        <v>2000000</v>
-      </c>
-      <c r="S4" s="21">
-        <f t="shared" si="3"/>
-        <v>2000000</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C4">
+        <f>3600/C3</f>
+        <v>90</v>
+      </c>
+      <c r="D4">
+        <v>90</v>
+      </c>
+      <c r="E4">
+        <v>90</v>
+      </c>
+      <c r="F4">
+        <v>90</v>
+      </c>
+      <c r="G4">
+        <v>90</v>
+      </c>
+      <c r="H4">
+        <v>90</v>
+      </c>
+      <c r="I4">
+        <v>90</v>
+      </c>
+      <c r="J4">
+        <v>90</v>
+      </c>
+      <c r="K4">
+        <v>90</v>
+      </c>
+      <c r="L4">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="23" t="s">
         <v>71</v>
       </c>
       <c r="B5" s="24">
         <v>7.5</v>
       </c>
-      <c r="D5" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="E5" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="F5" s="21">
-        <v>12</v>
-      </c>
-      <c r="G5" s="21">
-        <v>1</v>
-      </c>
-      <c r="H5" s="21">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="I5" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J5" s="21">
-        <f t="shared" ref="J5:S5" si="4">I5</f>
-        <v>112000</v>
-      </c>
-      <c r="K5" s="21">
-        <f t="shared" si="4"/>
-        <v>112000</v>
-      </c>
-      <c r="L5" s="21">
-        <f t="shared" si="4"/>
-        <v>112000</v>
-      </c>
-      <c r="M5" s="21">
-        <f t="shared" si="4"/>
-        <v>112000</v>
-      </c>
-      <c r="N5" s="21">
-        <f t="shared" si="4"/>
-        <v>112000</v>
-      </c>
-      <c r="O5" s="21">
-        <f t="shared" si="4"/>
-        <v>112000</v>
-      </c>
-      <c r="P5" s="21">
-        <f t="shared" si="4"/>
-        <v>112000</v>
-      </c>
-      <c r="Q5" s="21">
-        <f t="shared" si="4"/>
-        <v>112000</v>
-      </c>
-      <c r="R5" s="21">
-        <f t="shared" si="4"/>
-        <v>112000</v>
-      </c>
-      <c r="S5" s="21">
-        <f t="shared" si="4"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="69">
+        <v>7.5</v>
+      </c>
+      <c r="D5" s="69">
+        <v>7.5</v>
+      </c>
+      <c r="E5" s="69">
+        <v>7.5</v>
+      </c>
+      <c r="F5" s="69">
+        <v>7.5</v>
+      </c>
+      <c r="G5" s="69">
+        <v>7.5</v>
+      </c>
+      <c r="H5" s="69">
+        <v>7.5</v>
+      </c>
+      <c r="I5" s="69">
+        <v>7.5</v>
+      </c>
+      <c r="J5" s="69">
+        <v>7.5</v>
+      </c>
+      <c r="K5" s="69">
+        <v>7.5</v>
+      </c>
+      <c r="L5" s="69">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="23" t="s">
         <v>106</v>
       </c>
       <c r="B6" s="24">
         <v>2</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="F6" s="21">
-        <v>12</v>
-      </c>
-      <c r="G6" s="21">
+      <c r="C6" s="69">
         <v>1</v>
       </c>
-      <c r="H6" s="21">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="I6" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J6" s="21">
-        <f t="shared" ref="J6:S6" si="5">I6</f>
-        <v>112000</v>
-      </c>
-      <c r="K6" s="21">
-        <f t="shared" si="5"/>
-        <v>112000</v>
-      </c>
-      <c r="L6" s="21">
-        <f t="shared" si="5"/>
-        <v>112000</v>
-      </c>
-      <c r="M6" s="21">
-        <f t="shared" si="5"/>
-        <v>112000</v>
-      </c>
-      <c r="N6" s="21">
-        <f t="shared" si="5"/>
-        <v>112000</v>
-      </c>
-      <c r="O6" s="21">
-        <f t="shared" si="5"/>
-        <v>112000</v>
-      </c>
-      <c r="P6" s="21">
-        <f t="shared" si="5"/>
-        <v>112000</v>
-      </c>
-      <c r="Q6" s="21">
-        <f t="shared" si="5"/>
-        <v>112000</v>
-      </c>
-      <c r="R6" s="21">
-        <f t="shared" si="5"/>
-        <v>112000</v>
-      </c>
-      <c r="S6" s="21">
-        <f t="shared" si="5"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D6" s="69">
+        <v>1</v>
+      </c>
+      <c r="E6" s="69">
+        <v>1</v>
+      </c>
+      <c r="F6" s="69">
+        <v>1</v>
+      </c>
+      <c r="G6" s="69">
+        <v>1</v>
+      </c>
+      <c r="H6" s="69">
+        <v>1</v>
+      </c>
+      <c r="I6" s="69">
+        <v>1</v>
+      </c>
+      <c r="J6" s="69">
+        <v>1</v>
+      </c>
+      <c r="K6" s="69">
+        <v>1</v>
+      </c>
+      <c r="L6" s="69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="23" t="s">
         <v>109</v>
       </c>
       <c r="B7" s="24">
         <v>1</v>
       </c>
-      <c r="D7" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="E7" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="F7" s="21">
-        <v>12</v>
-      </c>
-      <c r="G7" s="21">
+      <c r="C7" s="69">
         <v>1</v>
       </c>
-      <c r="H7" s="21">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="I7" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J7" s="21">
-        <f t="shared" ref="J7:S7" si="6">I7</f>
-        <v>112000</v>
-      </c>
-      <c r="K7" s="21">
-        <f t="shared" si="6"/>
-        <v>112000</v>
-      </c>
-      <c r="L7" s="21">
-        <f t="shared" si="6"/>
-        <v>112000</v>
-      </c>
-      <c r="M7" s="21">
-        <f t="shared" si="6"/>
-        <v>112000</v>
-      </c>
-      <c r="N7" s="21">
-        <f t="shared" si="6"/>
-        <v>112000</v>
-      </c>
-      <c r="O7" s="21">
-        <f t="shared" si="6"/>
-        <v>112000</v>
-      </c>
-      <c r="P7" s="21">
-        <f t="shared" si="6"/>
-        <v>112000</v>
-      </c>
-      <c r="Q7" s="21">
-        <f t="shared" si="6"/>
-        <v>112000</v>
-      </c>
-      <c r="R7" s="21">
-        <f t="shared" si="6"/>
-        <v>112000</v>
-      </c>
-      <c r="S7" s="21">
-        <f t="shared" si="6"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D7" s="69">
+        <v>1</v>
+      </c>
+      <c r="E7" s="69">
+        <v>1</v>
+      </c>
+      <c r="F7" s="69">
+        <v>2</v>
+      </c>
+      <c r="G7" s="69">
+        <v>1</v>
+      </c>
+      <c r="H7" s="69">
+        <v>1</v>
+      </c>
+      <c r="I7" s="69">
+        <v>1</v>
+      </c>
+      <c r="J7" s="69">
+        <v>1</v>
+      </c>
+      <c r="K7" s="69">
+        <v>1</v>
+      </c>
+      <c r="L7" s="69">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="23" t="s">
         <v>112</v>
       </c>
       <c r="B8" s="24">
         <v>5</v>
       </c>
-      <c r="D8" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="F8" s="21">
-        <v>12</v>
-      </c>
-      <c r="G8" s="21">
-        <v>1</v>
-      </c>
-      <c r="H8" s="21">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="I8" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J8" s="21">
-        <f t="shared" ref="J8:S8" si="7">I8</f>
-        <v>112000</v>
-      </c>
-      <c r="K8" s="21">
-        <f t="shared" si="7"/>
-        <v>112000</v>
-      </c>
-      <c r="L8" s="21">
-        <f t="shared" si="7"/>
-        <v>112000</v>
-      </c>
-      <c r="M8" s="21">
-        <f t="shared" si="7"/>
-        <v>112000</v>
-      </c>
-      <c r="N8" s="21">
-        <f t="shared" si="7"/>
-        <v>112000</v>
-      </c>
-      <c r="O8" s="21">
-        <f t="shared" si="7"/>
-        <v>112000</v>
-      </c>
-      <c r="P8" s="21">
-        <f t="shared" si="7"/>
-        <v>112000</v>
-      </c>
-      <c r="Q8" s="21">
-        <f t="shared" si="7"/>
-        <v>112000</v>
-      </c>
-      <c r="R8" s="21">
-        <f t="shared" si="7"/>
-        <v>112000</v>
-      </c>
-      <c r="S8" s="21">
-        <f t="shared" si="7"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C8" s="69">
+        <v>5</v>
+      </c>
+      <c r="D8" s="69">
+        <v>5</v>
+      </c>
+      <c r="E8" s="69">
+        <v>5</v>
+      </c>
+      <c r="F8" s="69">
+        <v>5</v>
+      </c>
+      <c r="G8" s="69">
+        <v>5</v>
+      </c>
+      <c r="H8" s="69">
+        <v>5</v>
+      </c>
+      <c r="I8" s="69">
+        <v>5</v>
+      </c>
+      <c r="J8" s="69">
+        <v>6</v>
+      </c>
+      <c r="K8" s="69">
+        <v>6</v>
+      </c>
+      <c r="L8" s="69">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="23" t="s">
         <v>115</v>
       </c>
       <c r="B9" s="24">
         <v>4</v>
       </c>
-      <c r="D9" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="F9" s="21">
-        <v>12</v>
-      </c>
-      <c r="G9" s="21">
-        <v>1</v>
-      </c>
-      <c r="H9" s="21">
-        <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-      <c r="I9" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J9" s="21">
-        <f t="shared" ref="J9:S9" si="8">I9</f>
-        <v>112000</v>
-      </c>
-      <c r="K9" s="21">
-        <f t="shared" si="8"/>
-        <v>112000</v>
-      </c>
-      <c r="L9" s="21">
-        <f t="shared" si="8"/>
-        <v>112000</v>
-      </c>
-      <c r="M9" s="21">
-        <f t="shared" si="8"/>
-        <v>112000</v>
-      </c>
-      <c r="N9" s="21">
-        <f t="shared" si="8"/>
-        <v>112000</v>
-      </c>
-      <c r="O9" s="21">
-        <f t="shared" si="8"/>
-        <v>112000</v>
-      </c>
-      <c r="P9" s="21">
-        <f t="shared" si="8"/>
-        <v>112000</v>
-      </c>
-      <c r="Q9" s="21">
-        <f t="shared" si="8"/>
-        <v>112000</v>
-      </c>
-      <c r="R9" s="21">
-        <f t="shared" si="8"/>
-        <v>112000</v>
-      </c>
-      <c r="S9" s="21">
-        <f t="shared" si="8"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C9" s="69">
+        <v>4</v>
+      </c>
+      <c r="D9" s="69">
+        <v>4</v>
+      </c>
+      <c r="E9" s="69">
+        <v>4</v>
+      </c>
+      <c r="F9" s="69">
+        <v>4</v>
+      </c>
+      <c r="G9" s="69">
+        <v>4</v>
+      </c>
+      <c r="H9" s="69">
+        <v>4</v>
+      </c>
+      <c r="I9" s="69">
+        <v>4</v>
+      </c>
+      <c r="J9" s="69">
+        <v>4</v>
+      </c>
+      <c r="K9" s="69">
+        <v>4</v>
+      </c>
+      <c r="L9" s="69">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="33" t="s">
         <v>118</v>
       </c>
       <c r="B10" s="34">
         <v>12</v>
       </c>
-      <c r="D10" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="E10" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="F10" s="21">
+      <c r="C10" s="71">
         <v>12</v>
       </c>
-      <c r="G10" s="21">
-        <v>1</v>
-      </c>
-      <c r="H10" s="21">
-        <f t="shared" si="1"/>
+      <c r="D10" s="71">
         <v>12</v>
       </c>
-      <c r="I10" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J10" s="21">
-        <f t="shared" ref="J10:S10" si="9">I10</f>
-        <v>112000</v>
-      </c>
-      <c r="K10" s="21">
-        <f t="shared" si="9"/>
-        <v>112000</v>
-      </c>
-      <c r="L10" s="21">
-        <f t="shared" si="9"/>
-        <v>112000</v>
-      </c>
-      <c r="M10" s="21">
-        <f t="shared" si="9"/>
-        <v>112000</v>
-      </c>
-      <c r="N10" s="21">
-        <f t="shared" si="9"/>
-        <v>112000</v>
-      </c>
-      <c r="O10" s="21">
-        <f t="shared" si="9"/>
-        <v>112000</v>
-      </c>
-      <c r="P10" s="21">
-        <f t="shared" si="9"/>
-        <v>112000</v>
-      </c>
-      <c r="Q10" s="21">
-        <f t="shared" si="9"/>
-        <v>112000</v>
-      </c>
-      <c r="R10" s="21">
-        <f t="shared" si="9"/>
-        <v>112000</v>
-      </c>
-      <c r="S10" s="21">
-        <f t="shared" si="9"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="E10" s="71">
+        <v>12</v>
+      </c>
+      <c r="F10" s="71">
+        <v>12</v>
+      </c>
+      <c r="G10" s="71">
+        <v>12</v>
+      </c>
+      <c r="H10" s="71">
+        <v>12</v>
+      </c>
+      <c r="I10" s="71">
+        <v>12</v>
+      </c>
+      <c r="J10" s="71">
+        <v>12</v>
+      </c>
+      <c r="K10" s="71">
+        <v>12</v>
+      </c>
+      <c r="L10" s="71">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="35" t="s">
         <v>121</v>
       </c>
@@ -5299,479 +5070,2118 @@
         <f>B4*B5*B6*B7*B8*B9*B10</f>
         <v>30857.142857142855</v>
       </c>
-      <c r="D11" s="21" t="s">
+      <c r="C11" s="36">
+        <f>C4*C5*C6*C7*C8*C9*C10</f>
+        <v>162000</v>
+      </c>
+      <c r="D11" s="36">
+        <f t="shared" ref="D11:L11" si="0">D4*D5*D6*D7*D8*D9*D10</f>
+        <v>162000</v>
+      </c>
+      <c r="E11" s="36">
+        <f t="shared" si="0"/>
+        <v>162000</v>
+      </c>
+      <c r="F11" s="36">
+        <f t="shared" si="0"/>
+        <v>324000</v>
+      </c>
+      <c r="G11" s="36">
+        <f t="shared" si="0"/>
+        <v>162000</v>
+      </c>
+      <c r="H11" s="36">
+        <f t="shared" si="0"/>
+        <v>162000</v>
+      </c>
+      <c r="I11" s="36">
+        <f t="shared" si="0"/>
+        <v>162000</v>
+      </c>
+      <c r="J11" s="36">
+        <f t="shared" si="0"/>
+        <v>194400</v>
+      </c>
+      <c r="K11" s="36">
+        <f t="shared" si="0"/>
+        <v>194400</v>
+      </c>
+      <c r="L11" s="36">
+        <f t="shared" si="0"/>
+        <v>194400</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="14" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="15" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="16" spans="1:12" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="17" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E17" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F17" s="6">
+        <v>2025</v>
+      </c>
+      <c r="G17" s="6">
+        <f t="shared" ref="G17:P17" si="1">F17+1</f>
+        <v>2026</v>
+      </c>
+      <c r="H17" s="6">
+        <f t="shared" si="1"/>
+        <v>2027</v>
+      </c>
+      <c r="I17" s="6">
+        <f t="shared" si="1"/>
+        <v>2028</v>
+      </c>
+      <c r="J17" s="6">
+        <f t="shared" si="1"/>
+        <v>2029</v>
+      </c>
+      <c r="K17" s="6">
+        <f t="shared" si="1"/>
+        <v>2030</v>
+      </c>
+      <c r="L17" s="6">
+        <f t="shared" si="1"/>
+        <v>2031</v>
+      </c>
+      <c r="M17" s="6">
+        <f t="shared" si="1"/>
+        <v>2032</v>
+      </c>
+      <c r="N17" s="6">
+        <f t="shared" si="1"/>
+        <v>2033</v>
+      </c>
+      <c r="O17" s="6">
+        <f t="shared" si="1"/>
+        <v>2034</v>
+      </c>
+      <c r="P17" s="6">
+        <f t="shared" si="1"/>
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="21">
+        <v>60</v>
+      </c>
+      <c r="D18" s="21">
+        <v>6</v>
+      </c>
+      <c r="E18" s="21">
+        <f t="shared" ref="E18:E33" si="2">C18/D18</f>
+        <v>10</v>
+      </c>
+      <c r="F18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="G18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="H18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="I18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="J18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="K18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="L18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="M18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="N18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="O18" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="P18" s="21">
+        <v>2800000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B19" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="21">
+        <v>12</v>
+      </c>
+      <c r="D19" s="21">
+        <v>1</v>
+      </c>
+      <c r="E19" s="21">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F19" s="21">
+        <v>2400000</v>
+      </c>
+      <c r="G19" s="21">
+        <f t="shared" ref="G19:P19" si="3">F19</f>
+        <v>2400000</v>
+      </c>
+      <c r="H19" s="21">
+        <f t="shared" si="3"/>
+        <v>2400000</v>
+      </c>
+      <c r="I19" s="21">
+        <f t="shared" si="3"/>
+        <v>2400000</v>
+      </c>
+      <c r="J19" s="21">
+        <f t="shared" si="3"/>
+        <v>2400000</v>
+      </c>
+      <c r="K19" s="21">
+        <f t="shared" si="3"/>
+        <v>2400000</v>
+      </c>
+      <c r="L19" s="21">
+        <f t="shared" si="3"/>
+        <v>2400000</v>
+      </c>
+      <c r="M19" s="21">
+        <f t="shared" si="3"/>
+        <v>2400000</v>
+      </c>
+      <c r="N19" s="21">
+        <f t="shared" si="3"/>
+        <v>2400000</v>
+      </c>
+      <c r="O19" s="21">
+        <f t="shared" si="3"/>
+        <v>2400000</v>
+      </c>
+      <c r="P19" s="21">
+        <f t="shared" si="3"/>
+        <v>2400000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" s="21">
+        <v>12</v>
+      </c>
+      <c r="D20" s="21">
+        <v>1</v>
+      </c>
+      <c r="E20" s="21">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F20" s="21">
+        <v>2000000</v>
+      </c>
+      <c r="G20" s="21">
+        <f t="shared" ref="G20:P20" si="4">F20</f>
+        <v>2000000</v>
+      </c>
+      <c r="H20" s="21">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+      <c r="I20" s="21">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+      <c r="J20" s="21">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+      <c r="K20" s="21">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+      <c r="L20" s="21">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+      <c r="M20" s="21">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+      <c r="N20" s="21">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+      <c r="O20" s="21">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+      <c r="P20" s="21">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" s="21">
+        <v>12</v>
+      </c>
+      <c r="D21" s="21">
+        <v>1</v>
+      </c>
+      <c r="E21" s="21">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F21" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G21" s="21">
+        <f t="shared" ref="G21:P21" si="5">F21</f>
+        <v>112000</v>
+      </c>
+      <c r="H21" s="21">
+        <f t="shared" si="5"/>
+        <v>112000</v>
+      </c>
+      <c r="I21" s="21">
+        <f t="shared" si="5"/>
+        <v>112000</v>
+      </c>
+      <c r="J21" s="21">
+        <f t="shared" si="5"/>
+        <v>112000</v>
+      </c>
+      <c r="K21" s="21">
+        <f t="shared" si="5"/>
+        <v>112000</v>
+      </c>
+      <c r="L21" s="21">
+        <f t="shared" si="5"/>
+        <v>112000</v>
+      </c>
+      <c r="M21" s="21">
+        <f t="shared" si="5"/>
+        <v>112000</v>
+      </c>
+      <c r="N21" s="21">
+        <f t="shared" si="5"/>
+        <v>112000</v>
+      </c>
+      <c r="O21" s="21">
+        <f t="shared" si="5"/>
+        <v>112000</v>
+      </c>
+      <c r="P21" s="21">
+        <f t="shared" si="5"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="C22" s="21">
+        <v>12</v>
+      </c>
+      <c r="D22" s="21">
+        <v>1</v>
+      </c>
+      <c r="E22" s="21">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F22" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G22" s="21">
+        <f t="shared" ref="G22:P22" si="6">F22</f>
+        <v>112000</v>
+      </c>
+      <c r="H22" s="21">
+        <f t="shared" si="6"/>
+        <v>112000</v>
+      </c>
+      <c r="I22" s="21">
+        <f t="shared" si="6"/>
+        <v>112000</v>
+      </c>
+      <c r="J22" s="21">
+        <f t="shared" si="6"/>
+        <v>112000</v>
+      </c>
+      <c r="K22" s="21">
+        <f t="shared" si="6"/>
+        <v>112000</v>
+      </c>
+      <c r="L22" s="21">
+        <f t="shared" si="6"/>
+        <v>112000</v>
+      </c>
+      <c r="M22" s="21">
+        <f t="shared" si="6"/>
+        <v>112000</v>
+      </c>
+      <c r="N22" s="21">
+        <f t="shared" si="6"/>
+        <v>112000</v>
+      </c>
+      <c r="O22" s="21">
+        <f t="shared" si="6"/>
+        <v>112000</v>
+      </c>
+      <c r="P22" s="21">
+        <f t="shared" si="6"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="B23" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="C23" s="21">
+        <v>12</v>
+      </c>
+      <c r="D23" s="21">
+        <v>1</v>
+      </c>
+      <c r="E23" s="21">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F23" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G23" s="21">
+        <f t="shared" ref="G23:P23" si="7">F23</f>
+        <v>112000</v>
+      </c>
+      <c r="H23" s="21">
+        <f t="shared" si="7"/>
+        <v>112000</v>
+      </c>
+      <c r="I23" s="21">
+        <f t="shared" si="7"/>
+        <v>112000</v>
+      </c>
+      <c r="J23" s="21">
+        <f t="shared" si="7"/>
+        <v>112000</v>
+      </c>
+      <c r="K23" s="21">
+        <f t="shared" si="7"/>
+        <v>112000</v>
+      </c>
+      <c r="L23" s="21">
+        <f t="shared" si="7"/>
+        <v>112000</v>
+      </c>
+      <c r="M23" s="21">
+        <f t="shared" si="7"/>
+        <v>112000</v>
+      </c>
+      <c r="N23" s="21">
+        <f t="shared" si="7"/>
+        <v>112000</v>
+      </c>
+      <c r="O23" s="21">
+        <f t="shared" si="7"/>
+        <v>112000</v>
+      </c>
+      <c r="P23" s="21">
+        <f t="shared" si="7"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="C24" s="21">
+        <v>12</v>
+      </c>
+      <c r="D24" s="21">
+        <v>1</v>
+      </c>
+      <c r="E24" s="21">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F24" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G24" s="21">
+        <f t="shared" ref="G24:P24" si="8">F24</f>
+        <v>112000</v>
+      </c>
+      <c r="H24" s="21">
+        <f t="shared" si="8"/>
+        <v>112000</v>
+      </c>
+      <c r="I24" s="21">
+        <f t="shared" si="8"/>
+        <v>112000</v>
+      </c>
+      <c r="J24" s="21">
+        <f t="shared" si="8"/>
+        <v>112000</v>
+      </c>
+      <c r="K24" s="21">
+        <f t="shared" si="8"/>
+        <v>112000</v>
+      </c>
+      <c r="L24" s="21">
+        <f t="shared" si="8"/>
+        <v>112000</v>
+      </c>
+      <c r="M24" s="21">
+        <f t="shared" si="8"/>
+        <v>112000</v>
+      </c>
+      <c r="N24" s="21">
+        <f t="shared" si="8"/>
+        <v>112000</v>
+      </c>
+      <c r="O24" s="21">
+        <f t="shared" si="8"/>
+        <v>112000</v>
+      </c>
+      <c r="P24" s="21">
+        <f t="shared" si="8"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="B25" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C25" s="21">
+        <v>12</v>
+      </c>
+      <c r="D25" s="21">
+        <v>1</v>
+      </c>
+      <c r="E25" s="21">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F25" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G25" s="21">
+        <f t="shared" ref="G25:P25" si="9">F25</f>
+        <v>112000</v>
+      </c>
+      <c r="H25" s="21">
+        <f t="shared" si="9"/>
+        <v>112000</v>
+      </c>
+      <c r="I25" s="21">
+        <f t="shared" si="9"/>
+        <v>112000</v>
+      </c>
+      <c r="J25" s="21">
+        <f t="shared" si="9"/>
+        <v>112000</v>
+      </c>
+      <c r="K25" s="21">
+        <f t="shared" si="9"/>
+        <v>112000</v>
+      </c>
+      <c r="L25" s="21">
+        <f t="shared" si="9"/>
+        <v>112000</v>
+      </c>
+      <c r="M25" s="21">
+        <f t="shared" si="9"/>
+        <v>112000</v>
+      </c>
+      <c r="N25" s="21">
+        <f t="shared" si="9"/>
+        <v>112000</v>
+      </c>
+      <c r="O25" s="21">
+        <f t="shared" si="9"/>
+        <v>112000</v>
+      </c>
+      <c r="P25" s="21">
+        <f t="shared" si="9"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="C26" s="21">
+        <v>12</v>
+      </c>
+      <c r="D26" s="21">
+        <v>1</v>
+      </c>
+      <c r="E26" s="21">
+        <f t="shared" si="2"/>
+        <v>12</v>
+      </c>
+      <c r="F26" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G26" s="21">
+        <f t="shared" ref="G26:P26" si="10">F26</f>
+        <v>112000</v>
+      </c>
+      <c r="H26" s="21">
+        <f t="shared" si="10"/>
+        <v>112000</v>
+      </c>
+      <c r="I26" s="21">
+        <f t="shared" si="10"/>
+        <v>112000</v>
+      </c>
+      <c r="J26" s="21">
+        <f t="shared" si="10"/>
+        <v>112000</v>
+      </c>
+      <c r="K26" s="21">
+        <f t="shared" si="10"/>
+        <v>112000</v>
+      </c>
+      <c r="L26" s="21">
+        <f t="shared" si="10"/>
+        <v>112000</v>
+      </c>
+      <c r="M26" s="21">
+        <f t="shared" si="10"/>
+        <v>112000</v>
+      </c>
+      <c r="N26" s="21">
+        <f t="shared" si="10"/>
+        <v>112000</v>
+      </c>
+      <c r="O26" s="21">
+        <f t="shared" si="10"/>
+        <v>112000</v>
+      </c>
+      <c r="P26" s="21">
+        <f t="shared" si="10"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="E11" s="21" t="s">
+      <c r="B27" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="F11" s="21">
+      <c r="C27" s="21">
         <v>12</v>
       </c>
-      <c r="G11" s="21">
+      <c r="D27" s="21">
         <v>1</v>
       </c>
-      <c r="H11" s="21">
-        <f t="shared" si="1"/>
+      <c r="E27" s="21">
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="I11" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J11" s="21">
-        <f t="shared" ref="J11:S11" si="10">I11</f>
-        <v>112000</v>
-      </c>
-      <c r="K11" s="21">
-        <f t="shared" si="10"/>
-        <v>112000</v>
-      </c>
-      <c r="L11" s="21">
-        <f t="shared" si="10"/>
-        <v>112000</v>
-      </c>
-      <c r="M11" s="21">
-        <f t="shared" si="10"/>
-        <v>112000</v>
-      </c>
-      <c r="N11" s="21">
-        <f t="shared" si="10"/>
-        <v>112000</v>
-      </c>
-      <c r="O11" s="21">
-        <f t="shared" si="10"/>
-        <v>112000</v>
-      </c>
-      <c r="P11" s="21">
-        <f t="shared" si="10"/>
-        <v>112000</v>
-      </c>
-      <c r="Q11" s="21">
-        <f t="shared" si="10"/>
-        <v>112000</v>
-      </c>
-      <c r="R11" s="21">
-        <f t="shared" si="10"/>
-        <v>112000</v>
-      </c>
-      <c r="S11" s="21">
-        <f t="shared" si="10"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D12" s="21" t="s">
+      <c r="F27" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G27" s="21">
+        <f t="shared" ref="G27:P27" si="11">F27</f>
+        <v>112000</v>
+      </c>
+      <c r="H27" s="21">
+        <f t="shared" si="11"/>
+        <v>112000</v>
+      </c>
+      <c r="I27" s="21">
+        <f t="shared" si="11"/>
+        <v>112000</v>
+      </c>
+      <c r="J27" s="21">
+        <f t="shared" si="11"/>
+        <v>112000</v>
+      </c>
+      <c r="K27" s="21">
+        <f t="shared" si="11"/>
+        <v>112000</v>
+      </c>
+      <c r="L27" s="21">
+        <f t="shared" si="11"/>
+        <v>112000</v>
+      </c>
+      <c r="M27" s="21">
+        <f t="shared" si="11"/>
+        <v>112000</v>
+      </c>
+      <c r="N27" s="21">
+        <f t="shared" si="11"/>
+        <v>112000</v>
+      </c>
+      <c r="O27" s="21">
+        <f t="shared" si="11"/>
+        <v>112000</v>
+      </c>
+      <c r="P27" s="21">
+        <f t="shared" si="11"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="E12" s="21" t="s">
+      <c r="B28" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="F12" s="21">
+      <c r="C28" s="21">
         <v>12</v>
       </c>
-      <c r="G12" s="21">
+      <c r="D28" s="21">
         <v>1</v>
       </c>
-      <c r="H12" s="21">
-        <f t="shared" si="1"/>
+      <c r="E28" s="21">
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="I12" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J12" s="21">
-        <f t="shared" ref="J12:S12" si="11">I12</f>
-        <v>112000</v>
-      </c>
-      <c r="K12" s="21">
-        <f t="shared" si="11"/>
-        <v>112000</v>
-      </c>
-      <c r="L12" s="21">
-        <f t="shared" si="11"/>
-        <v>112000</v>
-      </c>
-      <c r="M12" s="21">
-        <f t="shared" si="11"/>
-        <v>112000</v>
-      </c>
-      <c r="N12" s="21">
-        <f t="shared" si="11"/>
-        <v>112000</v>
-      </c>
-      <c r="O12" s="21">
-        <f t="shared" si="11"/>
-        <v>112000</v>
-      </c>
-      <c r="P12" s="21">
-        <f t="shared" si="11"/>
-        <v>112000</v>
-      </c>
-      <c r="Q12" s="21">
-        <f t="shared" si="11"/>
-        <v>112000</v>
-      </c>
-      <c r="R12" s="21">
-        <f t="shared" si="11"/>
-        <v>112000</v>
-      </c>
-      <c r="S12" s="21">
-        <f t="shared" si="11"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D13" s="21" t="s">
+      <c r="F28" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G28" s="21">
+        <f t="shared" ref="G28:P28" si="12">F28</f>
+        <v>112000</v>
+      </c>
+      <c r="H28" s="21">
+        <f t="shared" si="12"/>
+        <v>112000</v>
+      </c>
+      <c r="I28" s="21">
+        <f t="shared" si="12"/>
+        <v>112000</v>
+      </c>
+      <c r="J28" s="21">
+        <f t="shared" si="12"/>
+        <v>112000</v>
+      </c>
+      <c r="K28" s="21">
+        <f t="shared" si="12"/>
+        <v>112000</v>
+      </c>
+      <c r="L28" s="21">
+        <f t="shared" si="12"/>
+        <v>112000</v>
+      </c>
+      <c r="M28" s="21">
+        <f t="shared" si="12"/>
+        <v>112000</v>
+      </c>
+      <c r="N28" s="21">
+        <f t="shared" si="12"/>
+        <v>112000</v>
+      </c>
+      <c r="O28" s="21">
+        <f t="shared" si="12"/>
+        <v>112000</v>
+      </c>
+      <c r="P28" s="21">
+        <f t="shared" si="12"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="E13" s="21" t="s">
+      <c r="B29" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="F13" s="21">
+      <c r="C29" s="21">
         <v>12</v>
       </c>
-      <c r="G13" s="21">
+      <c r="D29" s="21">
         <v>1</v>
       </c>
-      <c r="H13" s="21">
-        <f t="shared" si="1"/>
+      <c r="E29" s="21">
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="I13" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J13" s="21">
-        <f t="shared" ref="J13:S13" si="12">I13</f>
-        <v>112000</v>
-      </c>
-      <c r="K13" s="21">
-        <f t="shared" si="12"/>
-        <v>112000</v>
-      </c>
-      <c r="L13" s="21">
-        <f t="shared" si="12"/>
-        <v>112000</v>
-      </c>
-      <c r="M13" s="21">
-        <f t="shared" si="12"/>
-        <v>112000</v>
-      </c>
-      <c r="N13" s="21">
-        <f t="shared" si="12"/>
-        <v>112000</v>
-      </c>
-      <c r="O13" s="21">
-        <f t="shared" si="12"/>
-        <v>112000</v>
-      </c>
-      <c r="P13" s="21">
-        <f t="shared" si="12"/>
-        <v>112000</v>
-      </c>
-      <c r="Q13" s="21">
-        <f t="shared" si="12"/>
-        <v>112000</v>
-      </c>
-      <c r="R13" s="21">
-        <f t="shared" si="12"/>
-        <v>112000</v>
-      </c>
-      <c r="S13" s="21">
-        <f t="shared" si="12"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D14" s="10" t="s">
+      <c r="F29" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G29" s="21">
+        <f t="shared" ref="G29:P29" si="13">F29</f>
+        <v>112000</v>
+      </c>
+      <c r="H29" s="21">
+        <f t="shared" si="13"/>
+        <v>112000</v>
+      </c>
+      <c r="I29" s="21">
+        <f t="shared" si="13"/>
+        <v>112000</v>
+      </c>
+      <c r="J29" s="21">
+        <f t="shared" si="13"/>
+        <v>112000</v>
+      </c>
+      <c r="K29" s="21">
+        <f t="shared" si="13"/>
+        <v>112000</v>
+      </c>
+      <c r="L29" s="21">
+        <f t="shared" si="13"/>
+        <v>112000</v>
+      </c>
+      <c r="M29" s="21">
+        <f t="shared" si="13"/>
+        <v>112000</v>
+      </c>
+      <c r="N29" s="21">
+        <f t="shared" si="13"/>
+        <v>112000</v>
+      </c>
+      <c r="O29" s="21">
+        <f t="shared" si="13"/>
+        <v>112000</v>
+      </c>
+      <c r="P29" s="21">
+        <f t="shared" si="13"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="B30" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="F14" s="21">
+      <c r="C30" s="21">
         <v>12</v>
       </c>
-      <c r="G14" s="21">
+      <c r="D30" s="21">
         <v>1</v>
       </c>
-      <c r="H14" s="21">
-        <f t="shared" si="1"/>
+      <c r="E30" s="21">
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="I14" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J14" s="21">
-        <f t="shared" ref="J14:S14" si="13">I14</f>
-        <v>112000</v>
-      </c>
-      <c r="K14" s="21">
-        <f t="shared" si="13"/>
-        <v>112000</v>
-      </c>
-      <c r="L14" s="21">
-        <f t="shared" si="13"/>
-        <v>112000</v>
-      </c>
-      <c r="M14" s="21">
-        <f t="shared" si="13"/>
-        <v>112000</v>
-      </c>
-      <c r="N14" s="21">
-        <f t="shared" si="13"/>
-        <v>112000</v>
-      </c>
-      <c r="O14" s="21">
-        <f t="shared" si="13"/>
-        <v>112000</v>
-      </c>
-      <c r="P14" s="21">
-        <f t="shared" si="13"/>
-        <v>112000</v>
-      </c>
-      <c r="Q14" s="21">
-        <f t="shared" si="13"/>
-        <v>112000</v>
-      </c>
-      <c r="R14" s="21">
-        <f t="shared" si="13"/>
-        <v>112000</v>
-      </c>
-      <c r="S14" s="21">
-        <f t="shared" si="13"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="15" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D15" s="21" t="s">
+      <c r="F30" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G30" s="21">
+        <f t="shared" ref="G30:P30" si="14">F30</f>
+        <v>112000</v>
+      </c>
+      <c r="H30" s="21">
+        <f t="shared" si="14"/>
+        <v>112000</v>
+      </c>
+      <c r="I30" s="21">
+        <f t="shared" si="14"/>
+        <v>112000</v>
+      </c>
+      <c r="J30" s="21">
+        <f t="shared" si="14"/>
+        <v>112000</v>
+      </c>
+      <c r="K30" s="21">
+        <f t="shared" si="14"/>
+        <v>112000</v>
+      </c>
+      <c r="L30" s="21">
+        <f t="shared" si="14"/>
+        <v>112000</v>
+      </c>
+      <c r="M30" s="21">
+        <f t="shared" si="14"/>
+        <v>112000</v>
+      </c>
+      <c r="N30" s="21">
+        <f t="shared" si="14"/>
+        <v>112000</v>
+      </c>
+      <c r="O30" s="21">
+        <f t="shared" si="14"/>
+        <v>112000</v>
+      </c>
+      <c r="P30" s="21">
+        <f t="shared" si="14"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="B31" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="F15" s="21">
+      <c r="C31" s="21">
         <v>12</v>
       </c>
-      <c r="G15" s="21">
+      <c r="D31" s="21">
         <v>1</v>
       </c>
-      <c r="H15" s="21">
-        <f t="shared" si="1"/>
+      <c r="E31" s="21">
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="I15" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J15" s="21">
-        <f t="shared" ref="J15:S15" si="14">I15</f>
-        <v>112000</v>
-      </c>
-      <c r="K15" s="21">
-        <f t="shared" si="14"/>
-        <v>112000</v>
-      </c>
-      <c r="L15" s="21">
-        <f t="shared" si="14"/>
-        <v>112000</v>
-      </c>
-      <c r="M15" s="21">
-        <f t="shared" si="14"/>
-        <v>112000</v>
-      </c>
-      <c r="N15" s="21">
-        <f t="shared" si="14"/>
-        <v>112000</v>
-      </c>
-      <c r="O15" s="21">
-        <f t="shared" si="14"/>
-        <v>112000</v>
-      </c>
-      <c r="P15" s="21">
-        <f t="shared" si="14"/>
-        <v>112000</v>
-      </c>
-      <c r="Q15" s="21">
-        <f t="shared" si="14"/>
-        <v>112000</v>
-      </c>
-      <c r="R15" s="21">
-        <f t="shared" si="14"/>
-        <v>112000</v>
-      </c>
-      <c r="S15" s="21">
-        <f t="shared" si="14"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D16" s="21" t="s">
+      <c r="F31" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G31" s="21">
+        <f t="shared" ref="G31:P31" si="15">F31</f>
+        <v>112000</v>
+      </c>
+      <c r="H31" s="21">
+        <f t="shared" si="15"/>
+        <v>112000</v>
+      </c>
+      <c r="I31" s="21">
+        <f t="shared" si="15"/>
+        <v>112000</v>
+      </c>
+      <c r="J31" s="21">
+        <f t="shared" si="15"/>
+        <v>112000</v>
+      </c>
+      <c r="K31" s="21">
+        <f t="shared" si="15"/>
+        <v>112000</v>
+      </c>
+      <c r="L31" s="21">
+        <f t="shared" si="15"/>
+        <v>112000</v>
+      </c>
+      <c r="M31" s="21">
+        <f t="shared" si="15"/>
+        <v>112000</v>
+      </c>
+      <c r="N31" s="21">
+        <f t="shared" si="15"/>
+        <v>112000</v>
+      </c>
+      <c r="O31" s="21">
+        <f t="shared" si="15"/>
+        <v>112000</v>
+      </c>
+      <c r="P31" s="21">
+        <f t="shared" si="15"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="B32" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="F16" s="21">
+      <c r="C32" s="21">
         <v>12</v>
       </c>
-      <c r="G16" s="21">
+      <c r="D32" s="21">
         <v>1</v>
       </c>
-      <c r="H16" s="21">
-        <f t="shared" si="1"/>
+      <c r="E32" s="21">
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="I16" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J16" s="21">
-        <f t="shared" ref="J16:S16" si="15">I16</f>
-        <v>112000</v>
-      </c>
-      <c r="K16" s="21">
-        <f t="shared" si="15"/>
-        <v>112000</v>
-      </c>
-      <c r="L16" s="21">
-        <f t="shared" si="15"/>
-        <v>112000</v>
-      </c>
-      <c r="M16" s="21">
-        <f t="shared" si="15"/>
-        <v>112000</v>
-      </c>
-      <c r="N16" s="21">
-        <f t="shared" si="15"/>
-        <v>112000</v>
-      </c>
-      <c r="O16" s="21">
-        <f t="shared" si="15"/>
-        <v>112000</v>
-      </c>
-      <c r="P16" s="21">
-        <f t="shared" si="15"/>
-        <v>112000</v>
-      </c>
-      <c r="Q16" s="21">
-        <f t="shared" si="15"/>
-        <v>112000</v>
-      </c>
-      <c r="R16" s="21">
-        <f t="shared" si="15"/>
-        <v>112000</v>
-      </c>
-      <c r="S16" s="21">
-        <f t="shared" si="15"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="17" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="D17" s="21" t="s">
+      <c r="F32" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G32" s="21">
+        <f t="shared" ref="G32:P32" si="16">F32</f>
+        <v>112000</v>
+      </c>
+      <c r="H32" s="21">
+        <f t="shared" si="16"/>
+        <v>112000</v>
+      </c>
+      <c r="I32" s="21">
+        <f t="shared" si="16"/>
+        <v>112000</v>
+      </c>
+      <c r="J32" s="21">
+        <f t="shared" si="16"/>
+        <v>112000</v>
+      </c>
+      <c r="K32" s="21">
+        <f t="shared" si="16"/>
+        <v>112000</v>
+      </c>
+      <c r="L32" s="21">
+        <f t="shared" si="16"/>
+        <v>112000</v>
+      </c>
+      <c r="M32" s="21">
+        <f t="shared" si="16"/>
+        <v>112000</v>
+      </c>
+      <c r="N32" s="21">
+        <f t="shared" si="16"/>
+        <v>112000</v>
+      </c>
+      <c r="O32" s="21">
+        <f t="shared" si="16"/>
+        <v>112000</v>
+      </c>
+      <c r="P32" s="21">
+        <f t="shared" si="16"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="E17" s="21" t="s">
+      <c r="B33" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="F17" s="21">
+      <c r="C33" s="21">
         <v>120</v>
       </c>
-      <c r="G17" s="21">
+      <c r="D33" s="21">
         <v>3</v>
       </c>
-      <c r="H17" s="21">
-        <f t="shared" si="1"/>
+      <c r="E33" s="21">
+        <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="I17" s="21">
-        <v>112000</v>
-      </c>
-      <c r="J17" s="21">
-        <f t="shared" ref="J17:S17" si="16">I17</f>
-        <v>112000</v>
-      </c>
-      <c r="K17" s="21">
-        <f t="shared" si="16"/>
-        <v>112000</v>
-      </c>
-      <c r="L17" s="21">
-        <f t="shared" si="16"/>
-        <v>112000</v>
-      </c>
-      <c r="M17" s="21">
-        <f t="shared" si="16"/>
-        <v>112000</v>
-      </c>
-      <c r="N17" s="21">
-        <f t="shared" si="16"/>
-        <v>112000</v>
-      </c>
-      <c r="O17" s="21">
-        <f t="shared" si="16"/>
-        <v>112000</v>
-      </c>
-      <c r="P17" s="21">
-        <f t="shared" si="16"/>
-        <v>112000</v>
-      </c>
-      <c r="Q17" s="21">
-        <f t="shared" si="16"/>
-        <v>112000</v>
-      </c>
-      <c r="R17" s="21">
-        <f t="shared" si="16"/>
-        <v>112000</v>
-      </c>
-      <c r="S17" s="21">
-        <f t="shared" si="16"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="18" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="19" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="20" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="21" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="22" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="23" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="24" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="25" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="26" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="27" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="28" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="29" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="30" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="31" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="32" spans="4:19" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="36" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="37" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="38" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="39" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="40" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="41" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="42" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="43" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="44" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="45" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="46" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="47" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="48" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="52" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+      <c r="F33" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G33" s="21">
+        <f t="shared" ref="G33:P33" si="17">F33</f>
+        <v>112000</v>
+      </c>
+      <c r="H33" s="21">
+        <f t="shared" si="17"/>
+        <v>112000</v>
+      </c>
+      <c r="I33" s="21">
+        <f t="shared" si="17"/>
+        <v>112000</v>
+      </c>
+      <c r="J33" s="21">
+        <f t="shared" si="17"/>
+        <v>112000</v>
+      </c>
+      <c r="K33" s="21">
+        <f t="shared" si="17"/>
+        <v>112000</v>
+      </c>
+      <c r="L33" s="21">
+        <f t="shared" si="17"/>
+        <v>112000</v>
+      </c>
+      <c r="M33" s="21">
+        <f t="shared" si="17"/>
+        <v>112000</v>
+      </c>
+      <c r="N33" s="21">
+        <f t="shared" si="17"/>
+        <v>112000</v>
+      </c>
+      <c r="O33" s="21">
+        <f t="shared" si="17"/>
+        <v>112000</v>
+      </c>
+      <c r="P33" s="21">
+        <f t="shared" si="17"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="35" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C35" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D35" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="E35" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="F35" s="6">
+        <v>2025</v>
+      </c>
+      <c r="G35" s="6">
+        <f t="shared" ref="G35" si="18">F35+1</f>
+        <v>2026</v>
+      </c>
+      <c r="H35" s="6">
+        <f t="shared" ref="H35" si="19">G35+1</f>
+        <v>2027</v>
+      </c>
+      <c r="I35" s="6">
+        <f t="shared" ref="I35" si="20">H35+1</f>
+        <v>2028</v>
+      </c>
+      <c r="J35" s="6">
+        <f t="shared" ref="J35" si="21">I35+1</f>
+        <v>2029</v>
+      </c>
+      <c r="K35" s="6">
+        <f t="shared" ref="K35" si="22">J35+1</f>
+        <v>2030</v>
+      </c>
+      <c r="L35" s="6">
+        <f t="shared" ref="L35" si="23">K35+1</f>
+        <v>2031</v>
+      </c>
+      <c r="M35" s="6">
+        <f t="shared" ref="M35" si="24">L35+1</f>
+        <v>2032</v>
+      </c>
+      <c r="N35" s="6">
+        <f t="shared" ref="N35" si="25">M35+1</f>
+        <v>2033</v>
+      </c>
+      <c r="O35" s="6">
+        <f t="shared" ref="O35" si="26">N35+1</f>
+        <v>2034</v>
+      </c>
+      <c r="P35" s="6">
+        <f t="shared" ref="P35" si="27">O35+1</f>
+        <v>2035</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B36" s="21" t="s">
+        <v>39</v>
+      </c>
+      <c r="C36" s="21">
+        <v>60</v>
+      </c>
+      <c r="D36" s="21">
+        <v>6</v>
+      </c>
+      <c r="E36" s="21">
+        <f t="shared" ref="E36:F51" si="28">C36/D36</f>
+        <v>10</v>
+      </c>
+      <c r="F36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="G36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="H36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="I36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="J36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="K36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="L36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="M36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="N36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="O36" s="21">
+        <v>2800000</v>
+      </c>
+      <c r="P36" s="21">
+        <v>2800000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="C37" s="21">
+        <v>12</v>
+      </c>
+      <c r="D37" s="21">
+        <v>1</v>
+      </c>
+      <c r="E37" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F37" s="21">
+        <v>2400000</v>
+      </c>
+      <c r="G37" s="21">
+        <f t="shared" ref="G37:G51" si="29">F37</f>
+        <v>2400000</v>
+      </c>
+      <c r="H37" s="21">
+        <f t="shared" ref="H37:H51" si="30">G37</f>
+        <v>2400000</v>
+      </c>
+      <c r="I37" s="21">
+        <f t="shared" ref="I37:I51" si="31">H37</f>
+        <v>2400000</v>
+      </c>
+      <c r="J37" s="21">
+        <f t="shared" ref="J37:J51" si="32">I37</f>
+        <v>2400000</v>
+      </c>
+      <c r="K37" s="21">
+        <f t="shared" ref="K37:K51" si="33">J37</f>
+        <v>2400000</v>
+      </c>
+      <c r="L37" s="21">
+        <f t="shared" ref="L37:L51" si="34">K37</f>
+        <v>2400000</v>
+      </c>
+      <c r="M37" s="21">
+        <f t="shared" ref="M37:M51" si="35">L37</f>
+        <v>2400000</v>
+      </c>
+      <c r="N37" s="21">
+        <f t="shared" ref="N37:N51" si="36">M37</f>
+        <v>2400000</v>
+      </c>
+      <c r="O37" s="21">
+        <f t="shared" ref="O37:O51" si="37">N37</f>
+        <v>2400000</v>
+      </c>
+      <c r="P37" s="21">
+        <f t="shared" ref="P37:P51" si="38">O37</f>
+        <v>2400000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B38" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="C38" s="21">
+        <v>12</v>
+      </c>
+      <c r="D38" s="21">
+        <v>1</v>
+      </c>
+      <c r="E38" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F38" s="21">
+        <v>2000000</v>
+      </c>
+      <c r="G38" s="21">
+        <f t="shared" si="29"/>
+        <v>2000000</v>
+      </c>
+      <c r="H38" s="21">
+        <f t="shared" si="30"/>
+        <v>2000000</v>
+      </c>
+      <c r="I38" s="21">
+        <f t="shared" si="31"/>
+        <v>2000000</v>
+      </c>
+      <c r="J38" s="21">
+        <f t="shared" si="32"/>
+        <v>2000000</v>
+      </c>
+      <c r="K38" s="21">
+        <f t="shared" si="33"/>
+        <v>2000000</v>
+      </c>
+      <c r="L38" s="21">
+        <f t="shared" si="34"/>
+        <v>2000000</v>
+      </c>
+      <c r="M38" s="21">
+        <f t="shared" si="35"/>
+        <v>2000000</v>
+      </c>
+      <c r="N38" s="21">
+        <f t="shared" si="36"/>
+        <v>2000000</v>
+      </c>
+      <c r="O38" s="21">
+        <f t="shared" si="37"/>
+        <v>2000000</v>
+      </c>
+      <c r="P38" s="21">
+        <f t="shared" si="38"/>
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="B39" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="C39" s="21">
+        <v>12</v>
+      </c>
+      <c r="D39" s="21">
+        <v>1</v>
+      </c>
+      <c r="E39" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F39" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G39" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H39" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I39" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J39" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K39" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L39" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M39" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N39" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O39" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P39" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="B40" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="C40" s="21">
+        <v>12</v>
+      </c>
+      <c r="D40" s="21">
+        <v>1</v>
+      </c>
+      <c r="E40" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F40" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G40" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H40" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I40" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J40" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K40" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L40" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M40" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N40" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O40" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P40" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="B41" s="21" t="s">
+        <v>111</v>
+      </c>
+      <c r="C41" s="21">
+        <v>12</v>
+      </c>
+      <c r="D41" s="21">
+        <v>1</v>
+      </c>
+      <c r="E41" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F41" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G41" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H41" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I41" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J41" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K41" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L41" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M41" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N41" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O41" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P41" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A42" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="B42" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="C42" s="21">
+        <v>12</v>
+      </c>
+      <c r="D42" s="21">
+        <v>1</v>
+      </c>
+      <c r="E42" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F42" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G42" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H42" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I42" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J42" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K42" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L42" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M42" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N42" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O42" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P42" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="B43" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="C43" s="21">
+        <v>12</v>
+      </c>
+      <c r="D43" s="21">
+        <v>1</v>
+      </c>
+      <c r="E43" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F43" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G43" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H43" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I43" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J43" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K43" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L43" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M43" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N43" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O43" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P43" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B44" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="C44" s="21">
+        <v>12</v>
+      </c>
+      <c r="D44" s="21">
+        <v>1</v>
+      </c>
+      <c r="E44" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F44" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G44" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H44" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I44" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J44" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K44" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L44" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M44" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N44" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O44" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P44" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="B45" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="C45" s="21">
+        <v>12</v>
+      </c>
+      <c r="D45" s="21">
+        <v>1</v>
+      </c>
+      <c r="E45" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F45" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G45" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H45" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I45" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J45" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K45" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L45" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M45" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N45" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O45" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P45" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A46" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="B46" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="C46" s="21">
+        <v>12</v>
+      </c>
+      <c r="D46" s="21">
+        <v>1</v>
+      </c>
+      <c r="E46" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F46" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G46" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H46" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I46" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J46" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K46" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L46" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M46" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N46" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O46" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P46" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A47" s="21" t="s">
+        <v>126</v>
+      </c>
+      <c r="B47" s="21" t="s">
+        <v>127</v>
+      </c>
+      <c r="C47" s="21">
+        <v>12</v>
+      </c>
+      <c r="D47" s="21">
+        <v>1</v>
+      </c>
+      <c r="E47" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F47" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G47" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H47" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I47" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J47" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K47" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L47" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M47" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N47" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O47" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P47" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A48" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="B48" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="C48" s="21">
+        <v>12</v>
+      </c>
+      <c r="D48" s="21">
+        <v>1</v>
+      </c>
+      <c r="E48" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F48" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G48" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H48" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I48" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J48" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K48" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L48" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M48" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N48" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O48" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P48" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A49" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="B49" s="21" t="s">
+        <v>131</v>
+      </c>
+      <c r="C49" s="21">
+        <v>12</v>
+      </c>
+      <c r="D49" s="21">
+        <v>1</v>
+      </c>
+      <c r="E49" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F49" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G49" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H49" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I49" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J49" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K49" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L49" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M49" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N49" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O49" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P49" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="50" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A50" s="21" t="s">
+        <v>132</v>
+      </c>
+      <c r="B50" s="21" t="s">
+        <v>133</v>
+      </c>
+      <c r="C50" s="21">
+        <v>12</v>
+      </c>
+      <c r="D50" s="21">
+        <v>1</v>
+      </c>
+      <c r="E50" s="21">
+        <f t="shared" si="28"/>
+        <v>12</v>
+      </c>
+      <c r="F50" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G50" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H50" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I50" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J50" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K50" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L50" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M50" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N50" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O50" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P50" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="51" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A51" s="21" t="s">
+        <v>134</v>
+      </c>
+      <c r="B51" s="21" t="s">
+        <v>135</v>
+      </c>
+      <c r="C51" s="21">
+        <v>120</v>
+      </c>
+      <c r="D51" s="21">
+        <v>3</v>
+      </c>
+      <c r="E51" s="21">
+        <f t="shared" si="28"/>
+        <v>40</v>
+      </c>
+      <c r="F51" s="21">
+        <v>112000</v>
+      </c>
+      <c r="G51" s="21">
+        <f t="shared" si="29"/>
+        <v>112000</v>
+      </c>
+      <c r="H51" s="21">
+        <f t="shared" si="30"/>
+        <v>112000</v>
+      </c>
+      <c r="I51" s="21">
+        <f t="shared" si="31"/>
+        <v>112000</v>
+      </c>
+      <c r="J51" s="21">
+        <f t="shared" si="32"/>
+        <v>112000</v>
+      </c>
+      <c r="K51" s="21">
+        <f t="shared" si="33"/>
+        <v>112000</v>
+      </c>
+      <c r="L51" s="21">
+        <f t="shared" si="34"/>
+        <v>112000</v>
+      </c>
+      <c r="M51" s="21">
+        <f t="shared" si="35"/>
+        <v>112000</v>
+      </c>
+      <c r="N51" s="21">
+        <f t="shared" si="36"/>
+        <v>112000</v>
+      </c>
+      <c r="O51" s="21">
+        <f t="shared" si="37"/>
+        <v>112000</v>
+      </c>
+      <c r="P51" s="21">
+        <f t="shared" si="38"/>
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="52" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="65" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="67" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
fix: dont sum again the machinery
</commit_message>
<xml_diff>
--- a/Input_0.1.xlsx
+++ b/Input_0.1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\herna\Desktop\Repos\TecBooks_V2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{746121D2-7451-44DF-B741-4BD34FCB1C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF59ED4B-5499-46E3-9E6E-2B563F91DACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Premisas" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="656" uniqueCount="264">
   <si>
     <t>Producto:</t>
   </si>
@@ -1153,7 +1153,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="72">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1248,6 +1248,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4680,7 +4681,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="72" t="s">
         <v>3</v>
       </c>
       <c r="B1" s="6">
@@ -6143,1045 +6144,36 @@
       </c>
     </row>
     <row r="34" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="35" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="11" t="s">
-        <v>11</v>
-      </c>
-      <c r="B35" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>23</v>
-      </c>
-      <c r="E35" s="11" t="s">
-        <v>24</v>
-      </c>
-      <c r="F35" s="6">
-        <v>2025</v>
-      </c>
-      <c r="G35" s="6">
-        <f t="shared" ref="G35" si="18">F35+1</f>
-        <v>2026</v>
-      </c>
-      <c r="H35" s="6">
-        <f t="shared" ref="H35" si="19">G35+1</f>
-        <v>2027</v>
-      </c>
-      <c r="I35" s="6">
-        <f t="shared" ref="I35" si="20">H35+1</f>
-        <v>2028</v>
-      </c>
-      <c r="J35" s="6">
-        <f t="shared" ref="J35" si="21">I35+1</f>
-        <v>2029</v>
-      </c>
-      <c r="K35" s="6">
-        <f t="shared" ref="K35" si="22">J35+1</f>
-        <v>2030</v>
-      </c>
-      <c r="L35" s="6">
-        <f t="shared" ref="L35" si="23">K35+1</f>
-        <v>2031</v>
-      </c>
-      <c r="M35" s="6">
-        <f t="shared" ref="M35" si="24">L35+1</f>
-        <v>2032</v>
-      </c>
-      <c r="N35" s="6">
-        <f t="shared" ref="N35" si="25">M35+1</f>
-        <v>2033</v>
-      </c>
-      <c r="O35" s="6">
-        <f t="shared" ref="O35" si="26">N35+1</f>
-        <v>2034</v>
-      </c>
-      <c r="P35" s="6">
-        <f t="shared" ref="P35" si="27">O35+1</f>
-        <v>2035</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="B36" s="21" t="s">
-        <v>39</v>
-      </c>
-      <c r="C36" s="21">
-        <v>60</v>
-      </c>
-      <c r="D36" s="21">
-        <v>6</v>
-      </c>
-      <c r="E36" s="21">
-        <f t="shared" ref="E36:F51" si="28">C36/D36</f>
-        <v>10</v>
-      </c>
-      <c r="F36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="G36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="H36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="I36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="J36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="K36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="L36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="M36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="N36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="O36" s="21">
-        <v>2800000</v>
-      </c>
-      <c r="P36" s="21">
-        <v>2800000</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="21" t="s">
-        <v>52</v>
-      </c>
-      <c r="B37" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="C37" s="21">
-        <v>12</v>
-      </c>
-      <c r="D37" s="21">
-        <v>1</v>
-      </c>
-      <c r="E37" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F37" s="21">
-        <v>2400000</v>
-      </c>
-      <c r="G37" s="21">
-        <f t="shared" ref="G37:G51" si="29">F37</f>
-        <v>2400000</v>
-      </c>
-      <c r="H37" s="21">
-        <f t="shared" ref="H37:H51" si="30">G37</f>
-        <v>2400000</v>
-      </c>
-      <c r="I37" s="21">
-        <f t="shared" ref="I37:I51" si="31">H37</f>
-        <v>2400000</v>
-      </c>
-      <c r="J37" s="21">
-        <f t="shared" ref="J37:J51" si="32">I37</f>
-        <v>2400000</v>
-      </c>
-      <c r="K37" s="21">
-        <f t="shared" ref="K37:K51" si="33">J37</f>
-        <v>2400000</v>
-      </c>
-      <c r="L37" s="21">
-        <f t="shared" ref="L37:L51" si="34">K37</f>
-        <v>2400000</v>
-      </c>
-      <c r="M37" s="21">
-        <f t="shared" ref="M37:M51" si="35">L37</f>
-        <v>2400000</v>
-      </c>
-      <c r="N37" s="21">
-        <f t="shared" ref="N37:N51" si="36">M37</f>
-        <v>2400000</v>
-      </c>
-      <c r="O37" s="21">
-        <f t="shared" ref="O37:O51" si="37">N37</f>
-        <v>2400000</v>
-      </c>
-      <c r="P37" s="21">
-        <f t="shared" ref="P37:P51" si="38">O37</f>
-        <v>2400000</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="B38" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="C38" s="21">
-        <v>12</v>
-      </c>
-      <c r="D38" s="21">
-        <v>1</v>
-      </c>
-      <c r="E38" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F38" s="21">
-        <v>2000000</v>
-      </c>
-      <c r="G38" s="21">
-        <f t="shared" si="29"/>
-        <v>2000000</v>
-      </c>
-      <c r="H38" s="21">
-        <f t="shared" si="30"/>
-        <v>2000000</v>
-      </c>
-      <c r="I38" s="21">
-        <f t="shared" si="31"/>
-        <v>2000000</v>
-      </c>
-      <c r="J38" s="21">
-        <f t="shared" si="32"/>
-        <v>2000000</v>
-      </c>
-      <c r="K38" s="21">
-        <f t="shared" si="33"/>
-        <v>2000000</v>
-      </c>
-      <c r="L38" s="21">
-        <f t="shared" si="34"/>
-        <v>2000000</v>
-      </c>
-      <c r="M38" s="21">
-        <f t="shared" si="35"/>
-        <v>2000000</v>
-      </c>
-      <c r="N38" s="21">
-        <f t="shared" si="36"/>
-        <v>2000000</v>
-      </c>
-      <c r="O38" s="21">
-        <f t="shared" si="37"/>
-        <v>2000000</v>
-      </c>
-      <c r="P38" s="21">
-        <f t="shared" si="38"/>
-        <v>2000000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="B39" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="C39" s="21">
-        <v>12</v>
-      </c>
-      <c r="D39" s="21">
-        <v>1</v>
-      </c>
-      <c r="E39" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F39" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G39" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H39" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I39" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J39" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K39" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L39" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M39" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N39" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O39" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P39" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="B40" s="21" t="s">
-        <v>108</v>
-      </c>
-      <c r="C40" s="21">
-        <v>12</v>
-      </c>
-      <c r="D40" s="21">
-        <v>1</v>
-      </c>
-      <c r="E40" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F40" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G40" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H40" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I40" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J40" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K40" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L40" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M40" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N40" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O40" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P40" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="B41" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="C41" s="21">
-        <v>12</v>
-      </c>
-      <c r="D41" s="21">
-        <v>1</v>
-      </c>
-      <c r="E41" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F41" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G41" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H41" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I41" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J41" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K41" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L41" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M41" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N41" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O41" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P41" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="B42" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="C42" s="21">
-        <v>12</v>
-      </c>
-      <c r="D42" s="21">
-        <v>1</v>
-      </c>
-      <c r="E42" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F42" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G42" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H42" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I42" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J42" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K42" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L42" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M42" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N42" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O42" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P42" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="B43" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="C43" s="21">
-        <v>12</v>
-      </c>
-      <c r="D43" s="21">
-        <v>1</v>
-      </c>
-      <c r="E43" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F43" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G43" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H43" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I43" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J43" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K43" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L43" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M43" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N43" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O43" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P43" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="10" t="s">
-        <v>119</v>
-      </c>
-      <c r="B44" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="C44" s="21">
-        <v>12</v>
-      </c>
-      <c r="D44" s="21">
-        <v>1</v>
-      </c>
-      <c r="E44" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F44" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G44" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H44" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I44" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J44" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K44" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L44" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M44" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N44" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O44" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P44" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="B45" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="C45" s="21">
-        <v>12</v>
-      </c>
-      <c r="D45" s="21">
-        <v>1</v>
-      </c>
-      <c r="E45" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F45" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G45" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H45" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I45" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J45" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K45" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L45" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M45" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N45" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O45" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P45" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="B46" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="C46" s="21">
-        <v>12</v>
-      </c>
-      <c r="D46" s="21">
-        <v>1</v>
-      </c>
-      <c r="E46" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F46" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G46" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H46" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I46" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J46" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K46" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L46" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M46" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N46" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O46" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P46" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="B47" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="C47" s="21">
-        <v>12</v>
-      </c>
-      <c r="D47" s="21">
-        <v>1</v>
-      </c>
-      <c r="E47" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F47" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G47" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H47" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I47" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J47" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K47" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L47" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M47" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N47" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O47" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P47" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="10" t="s">
-        <v>128</v>
-      </c>
-      <c r="B48" s="21" t="s">
-        <v>129</v>
-      </c>
-      <c r="C48" s="21">
-        <v>12</v>
-      </c>
-      <c r="D48" s="21">
-        <v>1</v>
-      </c>
-      <c r="E48" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F48" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G48" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H48" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I48" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J48" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K48" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L48" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M48" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N48" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O48" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P48" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="B49" s="21" t="s">
-        <v>131</v>
-      </c>
-      <c r="C49" s="21">
-        <v>12</v>
-      </c>
-      <c r="D49" s="21">
-        <v>1</v>
-      </c>
-      <c r="E49" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F49" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G49" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H49" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I49" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J49" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K49" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L49" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M49" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N49" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O49" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P49" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="B50" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="C50" s="21">
-        <v>12</v>
-      </c>
-      <c r="D50" s="21">
-        <v>1</v>
-      </c>
-      <c r="E50" s="21">
-        <f t="shared" si="28"/>
-        <v>12</v>
-      </c>
-      <c r="F50" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G50" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H50" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I50" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J50" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K50" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L50" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M50" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N50" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O50" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P50" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="B51" s="21" t="s">
-        <v>135</v>
-      </c>
-      <c r="C51" s="21">
-        <v>120</v>
-      </c>
-      <c r="D51" s="21">
-        <v>3</v>
-      </c>
-      <c r="E51" s="21">
-        <f t="shared" si="28"/>
-        <v>40</v>
-      </c>
-      <c r="F51" s="21">
-        <v>112000</v>
-      </c>
-      <c r="G51" s="21">
-        <f t="shared" si="29"/>
-        <v>112000</v>
-      </c>
-      <c r="H51" s="21">
-        <f t="shared" si="30"/>
-        <v>112000</v>
-      </c>
-      <c r="I51" s="21">
-        <f t="shared" si="31"/>
-        <v>112000</v>
-      </c>
-      <c r="J51" s="21">
-        <f t="shared" si="32"/>
-        <v>112000</v>
-      </c>
-      <c r="K51" s="21">
-        <f t="shared" si="33"/>
-        <v>112000</v>
-      </c>
-      <c r="L51" s="21">
-        <f t="shared" si="34"/>
-        <v>112000</v>
-      </c>
-      <c r="M51" s="21">
-        <f t="shared" si="35"/>
-        <v>112000</v>
-      </c>
-      <c r="N51" s="21">
-        <f t="shared" si="36"/>
-        <v>112000</v>
-      </c>
-      <c r="O51" s="21">
-        <f t="shared" si="37"/>
-        <v>112000</v>
-      </c>
-      <c r="P51" s="21">
-        <f t="shared" si="38"/>
-        <v>112000</v>
-      </c>
-    </row>
-    <row r="52" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="53" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="54" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="55" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="56" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="57" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="58" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="61" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="62" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="63" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="64" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="35" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="36" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="37" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="38" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="40" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="41" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="42" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="43" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="44" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="45" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="46" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="47" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="48" spans="1:16" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="52" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="53" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="54" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="55" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="56" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="57" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="58" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="59" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="60" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="61" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="62" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="63" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
+    <row r="64" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="65" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="66" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="67" ht="14.25" customHeight="1" x14ac:dyDescent="0.3"/>

</xml_diff>